<commit_message>
Modificacion modelo vecm 20/10
</commit_message>
<xml_diff>
--- a/DATA/bd_tesis.xlsx
+++ b/DATA/bd_tesis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebasteitor\Desktop\MODELOS ECONOMETRICOS\DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gmendoza\Desktop\Repositorios\MODELOS-ECONOMETRICOS\DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{698DDAC1-CB59-4692-8DCE-AC2885A0299C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDA5DFA1-2885-4D52-99A5-7F8F41EC100D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10140" yWindow="0" windowWidth="17280" windowHeight="15585" xr2:uid="{3A7A9CE9-36D3-406C-942F-B2B38294790B}"/>
+    <workbookView xWindow="9660" yWindow="0" windowWidth="16005" windowHeight="15585" xr2:uid="{3A7A9CE9-36D3-406C-942F-B2B38294790B}"/>
   </bookViews>
   <sheets>
     <sheet name="bdat_tes" sheetId="9" r:id="rId1"/>
@@ -767,7 +767,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1254,7 +1254,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1741,7 +1741,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2228,7 +2228,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2715,7 +2715,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">

</xml_diff>

<commit_message>
nuevo modelo var con base 2
</commit_message>
<xml_diff>
--- a/DATA/bd_tesis.xlsx
+++ b/DATA/bd_tesis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29413"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gmendoza\Desktop\Repositorios\MODELOS-ECONOMETRICOS\DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebasteitor\Desktop\MODELOS ECONOMETRICOS\DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDA5DFA1-2885-4D52-99A5-7F8F41EC100D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B894BD2F-1527-4049-AF59-A5195D814991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9660" yWindow="0" windowWidth="16005" windowHeight="15585" xr2:uid="{3A7A9CE9-36D3-406C-942F-B2B38294790B}"/>
+    <workbookView xWindow="7155" yWindow="0" windowWidth="28695" windowHeight="15585" xr2:uid="{3A7A9CE9-36D3-406C-942F-B2B38294790B}"/>
   </bookViews>
   <sheets>
     <sheet name="bdat_tes" sheetId="9" r:id="rId1"/>
@@ -767,7 +767,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1254,7 +1254,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1741,7 +1741,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2228,7 +2228,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2715,7 +2715,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">

</xml_diff>